<commit_message>
Add bonus sociale to comparison
</commit_message>
<xml_diff>
--- a/esempio_confronto_corretto.xlsx
+++ b/esempio_confronto_corretto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/silviofornaro/Desktop/EnergiaSolidaleLast/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5856B289-D7A6-6042-B88F-111D0F7EDAB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7948C88B-6558-2A4A-A4F2-7081361C3E38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37500" yWindow="4580" windowWidth="29400" windowHeight="18440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9280" yWindow="2180" windowWidth="29400" windowHeight="18440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Confronto" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>nome cliente</t>
   </si>
@@ -84,6 +84,9 @@
   </si>
   <si>
     <t>TOTALE</t>
+  </si>
+  <si>
+    <t>Bonus sociale</t>
   </si>
 </sst>
 </file>
@@ -627,9 +630,21 @@
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
+      <c r="A12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B12" s="5">
+        <f>-21.6</f>
+        <v>-21.6</v>
+      </c>
+      <c r="C12" s="5">
+        <f>B12</f>
+        <v>-21.6</v>
+      </c>
+      <c r="D12" s="5">
+        <f>C12</f>
+        <v>-21.6</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -640,11 +655,11 @@
       </c>
       <c r="C13" s="9">
         <f>SUM(C4:C12)*B13/SUM(B4:B12)</f>
-        <v>10.273475719424461</v>
+        <v>11.079204545454544</v>
       </c>
       <c r="D13" s="9">
         <f>SUM(D4:D12)*B13/SUM(B4:B12)</f>
-        <v>2.2935836330935251</v>
+        <v>-4.4341520979020981</v>
       </c>
       <c r="G13" s="8"/>
     </row>
@@ -654,15 +669,15 @@
       </c>
       <c r="B14" s="5">
         <f>SUM(B4:B13)</f>
-        <v>53.900000000000006</v>
+        <v>32.300000000000004</v>
       </c>
       <c r="C14" s="5">
         <f t="shared" ref="C14:E14" si="0">SUM(C4:C13)</f>
-        <v>58.783475719424466</v>
+        <v>37.989204545454548</v>
       </c>
       <c r="D14" s="5">
         <f t="shared" si="0"/>
-        <v>13.123583633093524</v>
+        <v>-15.204152097902099</v>
       </c>
       <c r="E14" s="5">
         <f t="shared" si="0"/>

</xml_diff>